<commit_message>
docs: preserve Excel namespaces in downloadable workbooks
</commit_message>
<xml_diff>
--- a/doc/source/_static/data/supporting_files/Nomenclature_and_formulas.xlsx
+++ b/doc/source/_static/data/supporting_files/Nomenclature_and_formulas.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" ns1:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <ns1:AlternateContent>
@@ -686,7 +686,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" ns1:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0E+00"/>
     <numFmt numFmtId="165" formatCode="0.000"/>

</xml_diff>

<commit_message>
docs: preserve Excel namespaces in downloadable workbooks (#170)
</commit_message>
<xml_diff>
--- a/doc/source/_static/data/supporting_files/Nomenclature_and_formulas.xlsx
+++ b/doc/source/_static/data/supporting_files/Nomenclature_and_formulas.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" ns1:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <ns1:AlternateContent>
@@ -686,7 +686,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" ns1:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0E+00"/>
     <numFmt numFmtId="165" formatCode="0.000"/>

</xml_diff>